<commit_message>
chore: run 2026-03-16 15:29 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_16_03_2026.xlsx
+++ b/logs/Consolidado_16_03_2026.xlsx
@@ -695,10 +695,10 @@
         <v>71</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -15442,40 +15442,40 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>16/03/2026</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Naturia Invisible Dry Shampoo
 Champô Seco Invisível Lavanda Orgânica
 75 ml</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/naturia-invisible-dry-shampoo-7716350.html</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr"/>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr"/>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>7716350</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>20%</t>
         </is>

</xml_diff>